<commit_message>
updated mosipmaster xlsx file
Signed-off-by: Abhi <abhishek.shankarcs@gmail.com>
</commit_message>
<xml_diff>
--- a/mosip_master/xlsx/title.xlsx
+++ b/mosip_master/xlsx/title.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="54">
   <si>
     <t xml:space="preserve">lang_code</t>
   </si>
@@ -59,6 +59,15 @@
   </si>
   <si>
     <t xml:space="preserve">Female Title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MRSS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mrss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">others</t>
   </si>
   <si>
     <t xml:space="preserve">MIS</t>
@@ -305,7 +314,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr defaultColWidth="8.4296875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="23.6"/>
@@ -383,10 +392,10 @@
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>16</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>6</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>17</v>
@@ -400,16 +409,16 @@
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>9</v>
@@ -417,32 +426,32 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="4" t="s">
         <v>25</v>
       </c>
       <c r="E8" s="1" t="s">
@@ -451,16 +460,16 @@
     </row>
     <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>9</v>
@@ -468,32 +477,32 @@
     </row>
     <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
-        <v>30</v>
+    <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="s">
+        <v>26</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="5" t="s">
         <v>32</v>
       </c>
       <c r="E11" s="1" t="s">
@@ -502,16 +511,16 @@
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>9</v>
@@ -519,16 +528,16 @@
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>9</v>
@@ -536,10 +545,10 @@
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>38</v>
@@ -553,16 +562,16 @@
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>9</v>
@@ -570,16 +579,16 @@
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>9</v>
@@ -587,10 +596,10 @@
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>45</v>
@@ -604,16 +613,16 @@
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>9</v>
@@ -621,25 +630,42 @@
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E19" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E20" s="1" t="s">
         <v>9</v>
       </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>